<commit_message>
Adds 2025 year for CPI
</commit_message>
<xml_diff>
--- a/InputData/cpi.xlsx
+++ b/InputData/cpi.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us\InputData\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DanOBrien\Models\EPS\US\eps-us\InputData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21B39BD3-42AA-4DDE-BCD1-0F086876A133}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44EAE9FB-0F21-409F-9AAC-EAA7EA423475}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1995" yWindow="1785" windowWidth="24105" windowHeight="13785" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="79">
   <si>
     <t>CPI Consumer Price Index</t>
   </si>
@@ -265,6 +265,9 @@
   </si>
   <si>
     <t>2024............................................................................. .</t>
+  </si>
+  <si>
+    <t>2025............................................................................. .</t>
   </si>
 </sst>
 </file>
@@ -706,14 +709,17 @@
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B6" r:id="rId1" xr:uid="{F47F918C-32AA-4D20-82C5-543F093B1139}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId2"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:O62"/>
+  <dimension ref="A1:O64"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="14" max="14" width="10.5703125" customWidth="1"/>
@@ -2006,7 +2012,7 @@
         <v>1.8</v>
       </c>
       <c r="G57" s="6">
-        <f>$D$50/D57</f>
+        <f t="shared" ref="G57:G64" si="1">$D$50/D57</f>
         <v>0.89805481563188172</v>
       </c>
     </row>
@@ -2030,7 +2036,7 @@
         <v>1.2</v>
       </c>
       <c r="G58" s="6">
-        <f>$D$50/D58</f>
+        <f t="shared" si="1"/>
         <v>0.88711067149387013</v>
       </c>
     </row>
@@ -2054,7 +2060,7 @@
         <v>4.7</v>
       </c>
       <c r="G59" s="6">
-        <f>$D$50/D59</f>
+        <f t="shared" si="1"/>
         <v>0.84730412960844359</v>
       </c>
     </row>
@@ -2078,7 +2084,7 @@
         <v>8</v>
       </c>
       <c r="G60" s="6">
-        <f>$D$50/D60</f>
+        <f t="shared" si="1"/>
         <v>0.78452102304761584</v>
       </c>
     </row>
@@ -2096,7 +2102,7 @@
         <v>304.702</v>
       </c>
       <c r="G61" s="6">
-        <f>$D$50/D61</f>
+        <f t="shared" si="1"/>
         <v>0.75350342301658668</v>
       </c>
     </row>
@@ -2114,9 +2120,30 @@
         <v>313.68900000000002</v>
       </c>
       <c r="G62" s="6">
-        <f>$D$50/D62</f>
+        <f t="shared" si="1"/>
         <v>0.73191600598044548</v>
       </c>
+    </row>
+    <row r="63" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>78</v>
+      </c>
+      <c r="B63" s="8">
+        <v>320.13</v>
+      </c>
+      <c r="C63" s="8">
+        <v>324.16000000000003</v>
+      </c>
+      <c r="D63" s="8">
+        <v>321.96199999999999</v>
+      </c>
+      <c r="G63" s="6">
+        <f t="shared" si="1"/>
+        <v>0.71310900044104586</v>
+      </c>
+    </row>
+    <row r="64" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="G64" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Updates OCCF to 2025 USD
</commit_message>
<xml_diff>
--- a/InputData/cpi.xlsx
+++ b/InputData/cpi.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DanOBrien\Models\EPS\US\eps-us\InputData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44EAE9FB-0F21-409F-9AAC-EAA7EA423475}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFB328A3-8CB7-47C2-BBC4-A7946274395B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1995" yWindow="1785" windowWidth="24105" windowHeight="13785" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="81">
   <si>
     <t>CPI Consumer Price Index</t>
   </si>
@@ -268,6 +268,12 @@
   </si>
   <si>
     <t>2025............................................................................. .</t>
+  </si>
+  <si>
+    <t>Currency Year</t>
+  </si>
+  <si>
+    <t>Conversion</t>
   </si>
 </sst>
 </file>
@@ -657,7 +663,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
@@ -706,6 +712,23 @@
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>7</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>2025</v>
+      </c>
+      <c r="B14" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <f>Data!G63</f>
+        <v>0.71310900044104586</v>
+      </c>
+      <c r="B15" t="s">
+        <v>80</v>
       </c>
     </row>
   </sheetData>
@@ -2012,7 +2035,7 @@
         <v>1.8</v>
       </c>
       <c r="G57" s="6">
-        <f t="shared" ref="G57:G64" si="1">$D$50/D57</f>
+        <f t="shared" ref="G57:G63" si="1">$D$50/D57</f>
         <v>0.89805481563188172</v>
       </c>
     </row>

</xml_diff>